<commit_message>
Estructura por proyectos: cada desarrollo con sus actividades
40 carpetas en proyectos/, hoja PROYECTOS en Excel y export JSON.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PBI Desarrollos.xlsx
+++ b/PBI Desarrollos.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJECUCION DESAROLLO" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESARROLLOS LISTOS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LB" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROYECTOS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -8321,4 +8322,1955 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>% Avance</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Total actividades</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Realizadas</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Pendientes</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Próxima fecha</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Próximo entregable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REVISION ACTA PACC - FACC HW</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>revision-acta-pacc-facc-hw</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Módulo HW demostración funcional parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REVISION ACTA PACC - FACC SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>revision-acta-pacc-facc-servicios</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>14/05/2026</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Módulo servicios listo para prueba con actas reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REVISION ACTAS LIQUIDACION - HW</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>revision-actas-liquidacion-hw</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>14/05/2026</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Primera demostración checklist HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REVISION LINEA A LINEA HW</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>revision-linea-a-linea-hw</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Documento oportunidades automatización video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VALIDACION HW LINEA A LINEA NOKIA-LOCAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>validacion-hw-linea-a-linea-nokia-local</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Demo investigación revisión videos HW con IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GESTION ACCESOS EB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gestion-accesos-eb</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PROCESO</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Aplicación en pruebas funcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GESTION FIRMAS ACTAS DE LIQUIDACION</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gestion-firmas-actas-de-liquidacion</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PROCESO</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Entrada a producción tras aval Gestión de Riesgos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RADICACION ACTAS DE LIQUIDACION (FIRMAS)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>radicacion-actas-de-liquidacion-firmas</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PROCESO</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>27/03/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Versión estable en producción</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ACTUALIZACION POR SITIO EN PORTAL RF</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>actualizacion-por-sitio-en-portal-rf</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Flujo funcional actualización portal RF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>APROBACION ID TRABAJOS SITE ACCESS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>aprobacion-id-trabajos-site-access</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Flujo automatizado aprobaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ASIGNACION ACTIVIDAD ALIADO</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>asignacion-actividad-aliado</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Primera versión automatización asignación</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CREACION ID TRABAJOS SITE ACCESS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>creacion-id-trabajos-site-access</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Flujo automatizado creación IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CREACION USUARIO</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>creacion-usuario</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Flujo automatizado creación usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DESBLOQUEO USUARIO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>desbloqueo-usuario</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Flujo automatizado desbloqueo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GESTION DE OTS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gestion-de-ots</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Primera estructura automatización OTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GESTION PERMISOS ACCESO / VENTANAS MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>gestion-permisos-acceso-ventanas-mantenimiento</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Flujo automatizado permisos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTACION RUTA TX</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>implementacion-ruta-tx</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Documento flujo operativo TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PLANIFICACION MIGRACION / RUTA TX</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>planificacion-migracion-ruta-tx</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Documento planificación automatizable</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>REVISION FORMATOS FSE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>revision-formatos-fse</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Documento validaciones FSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>REVISION Y CONCEPTO DE TSS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>revision-y-concepto-de-tss</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Documento validaciones TSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO ENTREGA HITOS INSTALACION E INTEGRACION</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>seguimiento-entrega-hitos-instalacion-e-integracion</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Modelo control hitos integración</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO IMPLEMENTACION ACCESO</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>seguimiento-implementacion-acceso</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Flujo seguimiento accesos</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO IMPLEMENTACION TX</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>seguimiento-implementacion-tx</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Modelo seguimiento implementación</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO RFIC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>seguimiento-rfic</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Flujo control RFIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ACTA SISTEMATIZADA / CASOS DE BAJA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>acta-sistematizada-casos-de-baja</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>10</v>
+      </c>
+      <c r="F26" t="n">
+        <v>10</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>APP CHECK DOC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>app-check-doc</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>APP CHECK HW</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>app-check-hw</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" t="n">
+        <v>6</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>APP GESTION DE ACCESOS ESCALADOS</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>app-gestion-de-accesos-escalados</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>APP PENALIDADES</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>app-penalidades</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>20</v>
+      </c>
+      <c r="F30" t="n">
+        <v>20</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BI CONTRATOS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>bi-contratos</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BITACORAS DIRECTOS</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>bitacoras-directos</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CRONOGRAMA DESARROLLOS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>cronograma-desarrollos</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>13/05/2026</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ONAIR</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>onair</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PBI ACTAS DE BAJA</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>pbi-actas-de-baja</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CREACION ACTA SISTEMATIZADA HW BAJA</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>creacion-acta-sistematizada-hw-baja</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Acta HW baja operativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CREACION CASO DE RECOLECCION HW BAJA</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>creacion-caso-de-recoleccion-hw-baja</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Flujo funcional generación casos</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REVISION DOCUMENTACION DESINSTALACION / DESMONTE</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>revision-documentacion-desinstalacion-desmonte</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Primera versión funcional desmonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>REVISION DOCUMENTACION INSTALACION / MIGRACION</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>revision-documentacion-instalacion-migracion</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Primera versión funcional instalación</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>REVISION SITE FOLDER NOKIA-LOCAL</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>revision-site-folder-nokia-local</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Automatización revisión documental</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SOLICITUD ACCESO EB</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>solicitud-acceso-eb</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EN CURSO</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Flujo funcional solicitud accesos</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>